<commit_message>
update results in `UniteD-SRL - run.xlsx`
</commit_message>
<xml_diff>
--- a/results/UniteD-SRL - run.xlsx
+++ b/results/UniteD-SRL - run.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\vito\SRL\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A2E73F-E0C0-4A0E-A2A3-69D37B8BA1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF22AB8D-5115-4C14-850D-AFAD3BA3C1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8190" yWindow="165" windowWidth="22275" windowHeight="10365" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="42165" yWindow="2850" windowWidth="22275" windowHeight="10365" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dependency-based" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="21">
   <si>
     <t>English</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>google/gemma-3-1b-it</t>
+  </si>
+  <si>
+    <t>ONESHOT</t>
   </si>
 </sst>
 </file>
@@ -224,9 +227,6 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -246,6 +246,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -508,32 +511,32 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="I1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
       <c r="L1" s="2"/>
-      <c r="M1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="Q1" s="15" t="s">
+      <c r="M1" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="Q1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="U1" s="15" t="s">
+      <c r="R1" s="15"/>
+      <c r="S1" s="15"/>
+      <c r="U1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="Y1" s="15" t="s">
+      <c r="V1" s="15"/>
+      <c r="W1" s="15"/>
+      <c r="Y1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="Z1" s="16"/>
-      <c r="AA1" s="16"/>
+      <c r="Z1" s="15"/>
+      <c r="AA1" s="15"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="2"/>
       <c r="AD1" s="2"/>
@@ -553,44 +556,44 @@
       <c r="AR1" s="2"/>
     </row>
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="Q2" s="18" t="s">
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+      <c r="Q2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="U2" s="18" t="s">
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="U2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16"/>
-      <c r="Y2" s="18" t="s">
+      <c r="V2" s="15"/>
+      <c r="W2" s="15"/>
+      <c r="Y2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="16"/>
-      <c r="AA2" s="16"/>
+      <c r="Z2" s="15"/>
+      <c r="AA2" s="15"/>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
       <c r="AD2" s="2"/>
@@ -610,7 +613,7 @@
       <c r="AR2" s="2"/>
     </row>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="15"/>
       <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
@@ -698,22 +701,22 @@
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14" t="b">
+      <c r="B4" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H4" s="1"/>
@@ -786,22 +789,22 @@
     </row>
     <row r="5" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
-      <c r="B5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C5" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" s="14" t="b">
+      <c r="B5" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H5" s="1"/>
@@ -874,22 +877,22 @@
     </row>
     <row r="6" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
-      <c r="B6" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14" t="b">
+      <c r="B6" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H6" s="1"/>
@@ -962,22 +965,22 @@
     </row>
     <row r="7" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
-      <c r="B7" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E7" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="14" t="b">
+      <c r="B7" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H7" s="1"/>
@@ -1050,22 +1053,22 @@
     </row>
     <row r="8" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
-      <c r="B8" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E8" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14" t="b">
+      <c r="B8" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="13" t="b">
         <v>1</v>
       </c>
       <c r="H8" s="1"/>
@@ -1138,22 +1141,22 @@
     </row>
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
-      <c r="B9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" s="14" t="b">
+      <c r="B9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="13" t="b">
         <v>1</v>
       </c>
       <c r="H9" s="1"/>
@@ -1228,22 +1231,22 @@
       <c r="A10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" s="14" t="b">
+      <c r="B10" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H10" s="1"/>
@@ -1316,22 +1319,22 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
-      <c r="B11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C11" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" s="14" t="b">
+      <c r="B11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="13" t="b">
         <v>0</v>
       </c>
       <c r="I11">
@@ -1385,22 +1388,22 @@
     </row>
     <row r="12" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
-      <c r="B12" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C12" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" s="14" t="b">
+      <c r="B12" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="13" t="b">
         <v>0</v>
       </c>
       <c r="I12">
@@ -1454,22 +1457,22 @@
     </row>
     <row r="13" spans="1:44" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
-      <c r="B13" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="14" t="b">
+      <c r="B13" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="13" t="b">
         <v>0</v>
       </c>
       <c r="I13" s="6">
@@ -1523,22 +1526,22 @@
     </row>
     <row r="14" spans="1:44" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
-      <c r="B14" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E14" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F14" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" s="14" t="b">
+      <c r="B14" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" s="13" t="b">
         <v>1</v>
       </c>
       <c r="I14" s="6">
@@ -1592,22 +1595,22 @@
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
-      <c r="B15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="E15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G15" s="14" t="b">
+      <c r="B15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" s="13" t="b">
         <v>1</v>
       </c>
       <c r="I15" s="6">
@@ -1663,110 +1666,282 @@
       <c r="A16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="K16" s="10"/>
-      <c r="O16" s="10"/>
-      <c r="S16" s="10"/>
-      <c r="W16" s="10"/>
-      <c r="Y16" s="6" t="e">
+      <c r="B16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6">
+        <v>0</v>
+      </c>
+      <c r="J16" s="6">
+        <v>0</v>
+      </c>
+      <c r="K16" s="7">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6">
+        <v>0</v>
+      </c>
+      <c r="N16" s="6">
+        <v>0</v>
+      </c>
+      <c r="O16" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="6">
+        <v>0</v>
+      </c>
+      <c r="R16" s="6">
+        <v>0</v>
+      </c>
+      <c r="S16" s="7">
+        <v>0</v>
+      </c>
+      <c r="U16" s="6">
+        <v>0</v>
+      </c>
+      <c r="V16" s="6">
+        <v>0</v>
+      </c>
+      <c r="W16" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="6">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z16" s="6" t="e">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="6">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA16" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="7">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="12"/>
-      <c r="B17" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D17" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="E17" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G17" s="14" t="b">
+      <c r="B17" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" s="13" t="b">
         <v>1</v>
       </c>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="13"/>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="2"/>
-      <c r="W17" s="13"/>
-      <c r="X17" s="1"/>
-      <c r="Y17" s="6" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z17" s="6" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA17" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+      <c r="I17" s="6">
+        <v>17.18</v>
+      </c>
+      <c r="J17" s="6">
+        <v>7.58</v>
+      </c>
+      <c r="K17" s="7">
+        <v>10.52</v>
+      </c>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6">
+        <v>10.039999999999999</v>
+      </c>
+      <c r="N17" s="6">
+        <v>3.77</v>
+      </c>
+      <c r="O17" s="7">
+        <v>5.48</v>
+      </c>
+      <c r="Q17" s="6">
+        <v>19.420000000000002</v>
+      </c>
+      <c r="R17" s="6">
+        <v>8.6</v>
+      </c>
+      <c r="S17" s="7">
+        <v>11.92</v>
+      </c>
+      <c r="U17" s="6">
+        <v>13.54</v>
+      </c>
+      <c r="V17" s="6">
+        <v>6.31</v>
+      </c>
+      <c r="W17" s="7">
+        <v>8.61</v>
+      </c>
+      <c r="Y17" s="6">
+        <f t="shared" ref="Y17:Y19" si="6">AVERAGE(I17,M17,Q17,U17)</f>
+        <v>15.045</v>
+      </c>
+      <c r="Z17" s="6">
+        <f t="shared" ref="Z17:Z19" si="7">AVERAGE(J17,N17,R17,V17)</f>
+        <v>6.5649999999999995</v>
+      </c>
+      <c r="AA17" s="7">
+        <f t="shared" ref="AA17:AA19" si="8">AVERAGE(K17,O17,S17,W17)</f>
+        <v>9.1325000000000003</v>
       </c>
       <c r="AB17" s="2"/>
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
       <c r="AE17" s="1"/>
-      <c r="AF17" s="15"/>
-      <c r="AG17" s="16"/>
-      <c r="AH17" s="16"/>
-      <c r="AI17" s="16"/>
-      <c r="AJ17" s="16"/>
-      <c r="AK17" s="16"/>
+      <c r="AF17" s="14"/>
+      <c r="AG17" s="15"/>
+      <c r="AH17" s="15"/>
+      <c r="AI17" s="15"/>
+      <c r="AJ17" s="15"/>
+      <c r="AK17" s="15"/>
       <c r="AL17" s="1"/>
-      <c r="AM17" s="15"/>
-      <c r="AN17" s="16"/>
-      <c r="AO17" s="16"/>
-      <c r="AP17" s="16"/>
-      <c r="AQ17" s="16"/>
-      <c r="AR17" s="16"/>
+      <c r="AM17" s="14"/>
+      <c r="AN17" s="15"/>
+      <c r="AO17" s="15"/>
+      <c r="AP17" s="15"/>
+      <c r="AQ17" s="15"/>
+      <c r="AR17" s="15"/>
     </row>
-    <row r="18" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="18" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="6">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6">
+        <v>0</v>
+      </c>
+      <c r="N18" s="6">
+        <v>0</v>
+      </c>
+      <c r="O18" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="6">
+        <v>0</v>
+      </c>
+      <c r="R18" s="6">
+        <v>0</v>
+      </c>
+      <c r="S18" s="7">
+        <v>0</v>
+      </c>
+      <c r="U18" s="6">
+        <v>0</v>
+      </c>
+      <c r="V18" s="6">
+        <v>0</v>
+      </c>
+      <c r="W18" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Z18" s="6">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AA18" s="7">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C19" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="7"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="6"/>
+      <c r="S19" s="7"/>
+      <c r="U19" s="6"/>
+      <c r="V19" s="6"/>
+      <c r="W19" s="7"/>
+      <c r="Y19" s="6" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z19" s="6" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA19" s="7" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
     <row r="20" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="21" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2767,32 +2942,32 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="I1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
       <c r="L1" s="2"/>
-      <c r="M1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="Q1" s="15" t="s">
+      <c r="M1" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="Q1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="U1" s="15" t="s">
+      <c r="R1" s="15"/>
+      <c r="S1" s="15"/>
+      <c r="U1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="Y1" s="15" t="s">
+      <c r="V1" s="15"/>
+      <c r="W1" s="15"/>
+      <c r="Y1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="Z1" s="16"/>
-      <c r="AA1" s="16"/>
+      <c r="Z1" s="15"/>
+      <c r="AA1" s="15"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="2"/>
       <c r="AD1" s="2"/>
@@ -2812,44 +2987,44 @@
       <c r="AR1" s="2"/>
     </row>
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="Q2" s="18" t="s">
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+      <c r="Q2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="U2" s="18" t="s">
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="U2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16"/>
-      <c r="Y2" s="18" t="s">
+      <c r="V2" s="15"/>
+      <c r="W2" s="15"/>
+      <c r="Y2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="16"/>
-      <c r="AA2" s="16"/>
+      <c r="Z2" s="15"/>
+      <c r="AA2" s="15"/>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
       <c r="AD2" s="2"/>
@@ -2869,7 +3044,7 @@
       <c r="AR2" s="2"/>
     </row>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="15"/>
       <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
@@ -2957,22 +3132,22 @@
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14" t="b">
+      <c r="B4" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H4" s="1"/>
@@ -3045,22 +3220,22 @@
     </row>
     <row r="5" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
-      <c r="B5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C5" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" s="14" t="b">
+      <c r="B5" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H5" s="1"/>
@@ -3133,22 +3308,22 @@
     </row>
     <row r="6" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
-      <c r="B6" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14" t="b">
+      <c r="B6" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H6" s="1"/>
@@ -3221,22 +3396,22 @@
     </row>
     <row r="7" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
-      <c r="B7" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E7" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="14" t="b">
+      <c r="B7" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H7" s="1"/>
@@ -3246,11 +3421,11 @@
       <c r="J7" s="6">
         <v>66.98</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="6">
         <v>73.52</v>
       </c>
       <c r="L7" s="6"/>
-      <c r="M7" s="6">
+      <c r="M7" s="7">
         <v>78</v>
       </c>
       <c r="N7" s="6">
@@ -3309,22 +3484,22 @@
     </row>
     <row r="8" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
-      <c r="B8" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E8" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14" t="b">
+      <c r="B8" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="13" t="b">
         <v>1</v>
       </c>
       <c r="H8" s="1"/>
@@ -3397,22 +3572,22 @@
     </row>
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
-      <c r="B9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" s="14" t="b">
+      <c r="B9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="13" t="b">
         <v>1</v>
       </c>
       <c r="H9" s="1"/>
@@ -3487,22 +3662,22 @@
       <c r="A10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" s="14" t="b">
+      <c r="B10" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="13" t="b">
         <v>0</v>
       </c>
       <c r="H10" s="1"/>
@@ -3575,22 +3750,22 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
-      <c r="B11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C11" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" s="14" t="b">
+      <c r="B11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="13" t="b">
         <v>0</v>
       </c>
       <c r="I11">
@@ -3630,7 +3805,7 @@
         <v>15.7</v>
       </c>
       <c r="Y11" s="6">
-        <f t="shared" ref="Y11:AA17" si="1">AVERAGE(I11,M11,Q11,U11)</f>
+        <f t="shared" ref="Y11:AA19" si="1">AVERAGE(I11,M11,Q11,U11)</f>
         <v>56.392499999999998</v>
       </c>
       <c r="Z11" s="6">
@@ -3644,22 +3819,22 @@
     </row>
     <row r="12" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
-      <c r="B12" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C12" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" s="14" t="b">
+      <c r="B12" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="13" t="b">
         <v>0</v>
       </c>
       <c r="I12">
@@ -3713,22 +3888,22 @@
     </row>
     <row r="13" spans="1:44" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
-      <c r="B13" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="14" t="b">
+      <c r="B13" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="13" t="b">
         <v>0</v>
       </c>
       <c r="I13" s="6">
@@ -3782,22 +3957,22 @@
     </row>
     <row r="14" spans="1:44" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
-      <c r="B14" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E14" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F14" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" s="14" t="b">
+      <c r="B14" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" s="13" t="b">
         <v>1</v>
       </c>
       <c r="I14" s="6">
@@ -3851,22 +4026,22 @@
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
-      <c r="B15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="E15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G15" s="14" t="b">
+      <c r="B15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" s="13" t="b">
         <v>1</v>
       </c>
       <c r="I15" s="6">
@@ -3922,110 +4097,308 @@
       <c r="A16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="K16" s="10"/>
-      <c r="O16" s="10"/>
-      <c r="S16" s="10"/>
-      <c r="W16" s="10"/>
-      <c r="Y16" s="6" t="e">
+      <c r="B16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6">
+        <v>0</v>
+      </c>
+      <c r="J16" s="6">
+        <v>0</v>
+      </c>
+      <c r="K16" s="7">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6">
+        <v>0</v>
+      </c>
+      <c r="N16" s="6">
+        <v>0</v>
+      </c>
+      <c r="O16" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="6">
+        <v>0</v>
+      </c>
+      <c r="R16" s="6">
+        <v>0</v>
+      </c>
+      <c r="S16" s="7">
+        <v>0</v>
+      </c>
+      <c r="U16" s="6">
+        <v>0</v>
+      </c>
+      <c r="V16" s="6">
+        <v>0</v>
+      </c>
+      <c r="W16" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z16" s="6" t="e">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA16" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="7">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="12"/>
-      <c r="B17" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D17" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="E17" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G17" s="14" t="b">
+      <c r="B17" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" s="13" t="b">
         <v>1</v>
       </c>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="13"/>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="2"/>
-      <c r="W17" s="13"/>
-      <c r="X17" s="1"/>
-      <c r="Y17" s="6" t="e">
+      <c r="I17" s="6">
+        <v>5.63</v>
+      </c>
+      <c r="J17" s="6">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="K17" s="7">
+        <v>1.91</v>
+      </c>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6">
+        <v>10.48</v>
+      </c>
+      <c r="N17" s="6">
+        <v>1.79</v>
+      </c>
+      <c r="O17" s="7">
+        <v>3.05</v>
+      </c>
+      <c r="Q17" s="6">
+        <v>6.26</v>
+      </c>
+      <c r="R17" s="6">
+        <v>1.57</v>
+      </c>
+      <c r="S17" s="7">
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="U17" s="6">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="V17" s="6">
+        <v>1.08</v>
+      </c>
+      <c r="W17" s="7">
+        <v>1.74</v>
+      </c>
+      <c r="X17" s="19"/>
+      <c r="Y17" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z17" s="6" t="e">
+        <v>6.7224999999999993</v>
+      </c>
+      <c r="Z17" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA17" s="7" t="e">
+        <v>1.3975</v>
+      </c>
+      <c r="AA17" s="7">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>2.3024999999999998</v>
       </c>
       <c r="AB17" s="2"/>
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
       <c r="AE17" s="1"/>
-      <c r="AF17" s="15"/>
-      <c r="AG17" s="16"/>
-      <c r="AH17" s="16"/>
-      <c r="AI17" s="16"/>
-      <c r="AJ17" s="16"/>
-      <c r="AK17" s="16"/>
+      <c r="AF17" s="14"/>
+      <c r="AG17" s="15"/>
+      <c r="AH17" s="15"/>
+      <c r="AI17" s="15"/>
+      <c r="AJ17" s="15"/>
+      <c r="AK17" s="15"/>
       <c r="AL17" s="1"/>
-      <c r="AM17" s="15"/>
-      <c r="AN17" s="16"/>
-      <c r="AO17" s="16"/>
-      <c r="AP17" s="16"/>
-      <c r="AQ17" s="16"/>
-      <c r="AR17" s="16"/>
+      <c r="AM17" s="14"/>
+      <c r="AN17" s="15"/>
+      <c r="AO17" s="15"/>
+      <c r="AP17" s="15"/>
+      <c r="AQ17" s="15"/>
+      <c r="AR17" s="15"/>
     </row>
-    <row r="18" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="18" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="6">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6">
+        <v>0</v>
+      </c>
+      <c r="N18" s="6">
+        <v>0</v>
+      </c>
+      <c r="O18" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="6">
+        <v>0</v>
+      </c>
+      <c r="R18" s="6">
+        <v>0</v>
+      </c>
+      <c r="S18" s="7">
+        <v>0</v>
+      </c>
+      <c r="U18" s="6">
+        <v>0</v>
+      </c>
+      <c r="V18" s="6">
+        <v>0</v>
+      </c>
+      <c r="W18" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Z18" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AA18" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C19" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" s="6">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="J19" s="6">
+        <v>0.21</v>
+      </c>
+      <c r="K19" s="7">
+        <v>0.38</v>
+      </c>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6">
+        <v>5.73</v>
+      </c>
+      <c r="N19" s="6">
+        <v>0.85</v>
+      </c>
+      <c r="O19" s="7">
+        <v>1.48</v>
+      </c>
+      <c r="Q19" s="6">
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="R19" s="6">
+        <v>0.48</v>
+      </c>
+      <c r="S19" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="U19" s="6">
+        <v>1.84</v>
+      </c>
+      <c r="V19" s="6">
+        <v>0.37</v>
+      </c>
+      <c r="W19" s="7">
+        <v>0.62</v>
+      </c>
+      <c r="X19" s="19"/>
+      <c r="Y19" s="6">
+        <f t="shared" si="1"/>
+        <v>2.99</v>
+      </c>
+      <c r="Z19" s="6">
+        <f t="shared" si="1"/>
+        <v>0.47750000000000004</v>
+      </c>
+      <c r="AA19" s="7">
+        <f t="shared" si="1"/>
+        <v>0.82000000000000006</v>
+      </c>
+    </row>
     <row r="20" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="21" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4983,6 +5356,13 @@
     <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="AF17:AK17"/>
+    <mergeCell ref="AM17:AR17"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="U1:W1"/>
+    <mergeCell ref="Y1:AA1"/>
+    <mergeCell ref="M1:O1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="Q2:S2"/>
@@ -4990,13 +5370,6 @@
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="U2:W2"/>
-    <mergeCell ref="AF17:AK17"/>
-    <mergeCell ref="AM17:AR17"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="U1:W1"/>
-    <mergeCell ref="Y1:AA1"/>
-    <mergeCell ref="M1:O1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Result file updated and fix for entire dataset
</commit_message>
<xml_diff>
--- a/results/UniteD-SRL - run.xlsx
+++ b/results/UniteD-SRL - run.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lorpa\Documents\Università\Magistrale\Anno2\TESI\project\SRL\SRL\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32FA4499-A205-4082-8014-A1E5B1B9EB6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8BDAF93-6E5D-4031-9033-059C98D43366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dependency-based" sheetId="1" r:id="rId1"/>
@@ -1977,30 +1977,54 @@
       <c r="G20" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="7"/>
+      <c r="I20" s="6">
+        <v>10</v>
+      </c>
+      <c r="J20" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="K20" s="7">
+        <v>0.02</v>
+      </c>
       <c r="L20" s="6"/>
-      <c r="M20" s="6"/>
-      <c r="N20" s="6"/>
-      <c r="O20" s="7"/>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="6"/>
-      <c r="S20" s="7"/>
-      <c r="U20" s="6"/>
-      <c r="V20" s="6"/>
-      <c r="W20" s="7"/>
-      <c r="Y20" s="6" t="e">
+      <c r="M20" s="6">
+        <v>0</v>
+      </c>
+      <c r="N20" s="6">
+        <v>0</v>
+      </c>
+      <c r="O20" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="6">
+        <v>2.94</v>
+      </c>
+      <c r="R20" s="6">
+        <v>0</v>
+      </c>
+      <c r="S20" s="7">
+        <v>0.01</v>
+      </c>
+      <c r="U20" s="6">
+        <v>0</v>
+      </c>
+      <c r="V20" s="6">
+        <v>0</v>
+      </c>
+      <c r="W20" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="6">
         <f t="shared" ref="Y20:Y21" si="9">AVERAGE(I20,M20,Q20,U20)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z20" s="6" t="e">
+        <v>3.2349999999999999</v>
+      </c>
+      <c r="Z20" s="6">
         <f t="shared" ref="Z20:Z21" si="10">AVERAGE(J20,N20,R20,V20)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA20" s="7" t="e">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="AA20" s="7">
         <f t="shared" ref="AA20:AA21" si="11">AVERAGE(K20,O20,S20,W20)</f>
-        <v>#DIV/0!</v>
+        <v>7.4999999999999997E-3</v>
       </c>
     </row>
     <row r="21" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2023,30 +2047,54 @@
       <c r="G21" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="7"/>
+      <c r="I21" s="6">
+        <v>0</v>
+      </c>
+      <c r="J21" s="6">
+        <v>0</v>
+      </c>
+      <c r="K21" s="7">
+        <v>0</v>
+      </c>
       <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="7"/>
-      <c r="Q21" s="6"/>
-      <c r="R21" s="6"/>
-      <c r="S21" s="7"/>
-      <c r="U21" s="6"/>
-      <c r="V21" s="6"/>
-      <c r="W21" s="7"/>
-      <c r="Y21" s="6" t="e">
+      <c r="M21" s="6">
+        <v>3.06</v>
+      </c>
+      <c r="N21" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="O21" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="Q21" s="6">
+        <v>0</v>
+      </c>
+      <c r="R21" s="6">
+        <v>0</v>
+      </c>
+      <c r="S21" s="7">
+        <v>0</v>
+      </c>
+      <c r="U21" s="6">
+        <v>0</v>
+      </c>
+      <c r="V21" s="6">
+        <v>0</v>
+      </c>
+      <c r="W21" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="6">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z21" s="6" t="e">
+        <v>0.76500000000000001</v>
+      </c>
+      <c r="Z21" s="6">
         <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA21" s="7" t="e">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="AA21" s="7">
         <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+        <v>5.0000000000000001E-3</v>
       </c>
     </row>
     <row r="22" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2071,35 +2119,320 @@
       <c r="G22" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="7"/>
+      <c r="I22" s="6">
+        <v>4.05</v>
+      </c>
+      <c r="J22" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="K22" s="7">
+        <v>0.19</v>
+      </c>
       <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="7"/>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="7"/>
-      <c r="U22" s="6"/>
-      <c r="V22" s="6"/>
-      <c r="W22" s="7"/>
-      <c r="Y22" s="6" t="e">
-        <f t="shared" ref="Y22" si="12">AVERAGE(I22,M22,Q22,U22)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z22" s="6" t="e">
-        <f t="shared" ref="Z22" si="13">AVERAGE(J22,N22,R22,V22)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA22" s="7" t="e">
-        <f t="shared" ref="AA22" si="14">AVERAGE(K22,O22,S22,W22)</f>
-        <v>#DIV/0!</v>
+      <c r="M22" s="6">
+        <v>7.03</v>
+      </c>
+      <c r="N22" s="6">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O22" s="7">
+        <v>0.27</v>
+      </c>
+      <c r="Q22" s="6">
+        <v>5.43</v>
+      </c>
+      <c r="R22" s="6">
+        <v>0.08</v>
+      </c>
+      <c r="S22" s="7">
+        <v>0.17</v>
+      </c>
+      <c r="U22" s="6">
+        <v>3.22</v>
+      </c>
+      <c r="V22" s="6">
+        <v>0</v>
+      </c>
+      <c r="W22" s="7">
+        <v>0.01</v>
+      </c>
+      <c r="Y22" s="6">
+        <f t="shared" ref="Y22:Y25" si="12">AVERAGE(I22,M22,Q22,U22)</f>
+        <v>4.9324999999999992</v>
+      </c>
+      <c r="Z22" s="6">
+        <f t="shared" ref="Z22:Z25" si="13">AVERAGE(J22,N22,R22,V22)</f>
+        <v>0.08</v>
+      </c>
+      <c r="AA22" s="7">
+        <f t="shared" ref="AA22:AA25" si="14">AVERAGE(K22,O22,S22,W22)</f>
+        <v>0.16</v>
       </c>
     </row>
-    <row r="23" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="12"/>
+      <c r="B23" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C23" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" s="1"/>
+      <c r="I23" s="6">
+        <v>5.82</v>
+      </c>
+      <c r="J23" s="6">
+        <v>0.31</v>
+      </c>
+      <c r="K23" s="7">
+        <v>0.59</v>
+      </c>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6">
+        <v>4.8</v>
+      </c>
+      <c r="N23" s="6">
+        <v>0.22</v>
+      </c>
+      <c r="O23" s="7">
+        <v>0.42</v>
+      </c>
+      <c r="Q23" s="6">
+        <v>14.6</v>
+      </c>
+      <c r="R23" s="6">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="S23" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U23" s="6">
+        <v>20</v>
+      </c>
+      <c r="V23" s="6">
+        <v>0.12</v>
+      </c>
+      <c r="W23" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="Y23" s="6">
+        <f t="shared" si="12"/>
+        <v>11.305</v>
+      </c>
+      <c r="Z23" s="6">
+        <f t="shared" si="13"/>
+        <v>0.30500000000000005</v>
+      </c>
+      <c r="AA23" s="7">
+        <f t="shared" si="14"/>
+        <v>0.59000000000000008</v>
+      </c>
+      <c r="AB23" s="6"/>
+      <c r="AC23" s="6"/>
+      <c r="AD23" s="6"/>
+      <c r="AE23" s="6"/>
+      <c r="AF23" s="6"/>
+      <c r="AG23" s="6"/>
+      <c r="AH23" s="6"/>
+      <c r="AI23" s="6"/>
+      <c r="AJ23" s="6"/>
+      <c r="AK23" s="6"/>
+      <c r="AL23" s="6"/>
+      <c r="AM23" s="6"/>
+      <c r="AN23" s="6"/>
+      <c r="AO23" s="6"/>
+      <c r="AP23" s="6"/>
+      <c r="AQ23" s="6"/>
+      <c r="AR23" s="6"/>
+    </row>
+    <row r="24" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="12"/>
+      <c r="B24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" s="1"/>
+      <c r="I24" s="6">
+        <v>3.73</v>
+      </c>
+      <c r="J24" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="K24" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6">
+        <v>3.82</v>
+      </c>
+      <c r="N24" s="6">
+        <v>0.49</v>
+      </c>
+      <c r="O24" s="7">
+        <v>0.88</v>
+      </c>
+      <c r="Q24" s="6">
+        <v>7.97</v>
+      </c>
+      <c r="R24" s="6">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="S24" s="7">
+        <v>1.92</v>
+      </c>
+      <c r="U24" s="6">
+        <v>8.9700000000000006</v>
+      </c>
+      <c r="V24" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="W24" s="7">
+        <v>1.32</v>
+      </c>
+      <c r="Y24" s="6">
+        <f t="shared" si="12"/>
+        <v>6.1225000000000005</v>
+      </c>
+      <c r="Z24" s="6">
+        <f t="shared" si="13"/>
+        <v>0.75</v>
+      </c>
+      <c r="AA24" s="7">
+        <f t="shared" si="14"/>
+        <v>1.33</v>
+      </c>
+      <c r="AB24" s="6"/>
+      <c r="AC24" s="6"/>
+      <c r="AD24" s="6"/>
+      <c r="AE24" s="6"/>
+      <c r="AF24" s="6"/>
+      <c r="AG24" s="6"/>
+      <c r="AH24" s="6"/>
+      <c r="AI24" s="6"/>
+      <c r="AJ24" s="6"/>
+      <c r="AK24" s="6"/>
+      <c r="AL24" s="6"/>
+      <c r="AM24" s="6"/>
+      <c r="AN24" s="6"/>
+      <c r="AO24" s="6"/>
+      <c r="AP24" s="6"/>
+      <c r="AQ24" s="6"/>
+      <c r="AR24" s="6"/>
+    </row>
+    <row r="25" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" s="1"/>
+      <c r="I25" s="6">
+        <v>8.5500000000000007</v>
+      </c>
+      <c r="J25" s="6">
+        <v>1.29</v>
+      </c>
+      <c r="K25" s="7">
+        <v>2.2400000000000002</v>
+      </c>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6">
+        <v>4.4800000000000004</v>
+      </c>
+      <c r="N25" s="6">
+        <v>0.24</v>
+      </c>
+      <c r="O25" s="7">
+        <v>0.47</v>
+      </c>
+      <c r="Q25" s="6">
+        <v>14.55</v>
+      </c>
+      <c r="R25" s="6">
+        <v>1.82</v>
+      </c>
+      <c r="S25" s="7">
+        <v>3.24</v>
+      </c>
+      <c r="U25" s="6">
+        <v>15.37</v>
+      </c>
+      <c r="V25" s="6">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="W25" s="7">
+        <v>2.08</v>
+      </c>
+      <c r="Y25" s="6">
+        <f t="shared" si="12"/>
+        <v>10.737500000000001</v>
+      </c>
+      <c r="Z25" s="6">
+        <f t="shared" si="13"/>
+        <v>1.1175000000000002</v>
+      </c>
+      <c r="AA25" s="7">
+        <f t="shared" si="14"/>
+        <v>2.0075000000000003</v>
+      </c>
+      <c r="AB25" s="6"/>
+      <c r="AC25" s="6"/>
+      <c r="AD25" s="6"/>
+      <c r="AE25" s="6"/>
+      <c r="AF25" s="6"/>
+      <c r="AG25" s="6"/>
+      <c r="AH25" s="6"/>
+      <c r="AI25" s="6"/>
+      <c r="AJ25" s="6"/>
+      <c r="AK25" s="6"/>
+      <c r="AL25" s="6"/>
+      <c r="AM25" s="6"/>
+      <c r="AN25" s="6"/>
+      <c r="AO25" s="6"/>
+      <c r="AP25" s="6"/>
+      <c r="AQ25" s="6"/>
+      <c r="AR25" s="6"/>
+    </row>
     <row r="26" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3957,7 +4290,7 @@
         <v>15.7</v>
       </c>
       <c r="Y11" s="6">
-        <f t="shared" ref="Y11:AA22" si="1">AVERAGE(I11,M11,Q11,U11)</f>
+        <f t="shared" ref="Y11:AA25" si="1">AVERAGE(I11,M11,Q11,U11)</f>
         <v>56.392499999999998</v>
       </c>
       <c r="Z11" s="6">
@@ -4573,30 +4906,54 @@
       <c r="G20" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="7"/>
+      <c r="I20" s="6">
+        <v>13.47</v>
+      </c>
+      <c r="J20" s="6">
+        <v>0.08</v>
+      </c>
+      <c r="K20" s="7">
+        <v>0.16</v>
+      </c>
       <c r="L20" s="6"/>
-      <c r="M20" s="6"/>
-      <c r="N20" s="6"/>
-      <c r="O20" s="7"/>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="6"/>
-      <c r="S20" s="7"/>
-      <c r="U20" s="6"/>
-      <c r="V20" s="6"/>
-      <c r="W20" s="7"/>
-      <c r="Y20" s="6" t="e">
+      <c r="M20" s="6">
+        <v>18.59</v>
+      </c>
+      <c r="N20" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="O20" s="7">
+        <v>0.09</v>
+      </c>
+      <c r="Q20" s="6">
+        <v>9.7799999999999994</v>
+      </c>
+      <c r="R20" s="6">
+        <v>0.02</v>
+      </c>
+      <c r="S20" s="7">
+        <v>0.04</v>
+      </c>
+      <c r="U20" s="6">
+        <v>14.28</v>
+      </c>
+      <c r="V20" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="W20" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="Y20" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z20" s="6" t="e">
+        <v>14.030000000000001</v>
+      </c>
+      <c r="Z20" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA20" s="7" t="e">
+        <v>3.7499999999999999E-2</v>
+      </c>
+      <c r="AA20" s="7">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>7.7499999999999999E-2</v>
       </c>
     </row>
     <row r="21" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4619,30 +4976,54 @@
       <c r="G21" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="7"/>
+      <c r="I21" s="6">
+        <v>8.83</v>
+      </c>
+      <c r="J21" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="K21" s="7">
+        <v>0.03</v>
+      </c>
       <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="7"/>
-      <c r="Q21" s="6"/>
-      <c r="R21" s="6"/>
-      <c r="S21" s="7"/>
-      <c r="U21" s="6"/>
-      <c r="V21" s="6"/>
-      <c r="W21" s="7"/>
-      <c r="Y21" s="6" t="e">
+      <c r="M21" s="6">
+        <v>13.85</v>
+      </c>
+      <c r="N21" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="O21" s="7">
+        <v>0.09</v>
+      </c>
+      <c r="Q21" s="6">
+        <v>16.66</v>
+      </c>
+      <c r="R21" s="6">
+        <v>0.06</v>
+      </c>
+      <c r="S21" s="7">
+        <v>0.12</v>
+      </c>
+      <c r="U21" s="6">
+        <v>14.62</v>
+      </c>
+      <c r="V21" s="6">
+        <v>0.09</v>
+      </c>
+      <c r="W21" s="7">
+        <v>0.19</v>
+      </c>
+      <c r="Y21" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z21" s="6" t="e">
+        <v>13.49</v>
+      </c>
+      <c r="Z21" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA21" s="7" t="e">
+        <v>0.05</v>
+      </c>
+      <c r="AA21" s="7">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>0.1075</v>
       </c>
     </row>
     <row r="22" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4667,35 +5048,320 @@
       <c r="G22" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="7"/>
+      <c r="I22" s="6">
+        <v>10.45</v>
+      </c>
+      <c r="J22" s="6">
+        <v>0.34</v>
+      </c>
+      <c r="K22" s="7">
+        <v>0.66</v>
+      </c>
       <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="7"/>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="7"/>
-      <c r="U22" s="6"/>
-      <c r="V22" s="6"/>
-      <c r="W22" s="7"/>
-      <c r="Y22" s="6" t="e">
+      <c r="M22" s="6">
+        <v>6.02</v>
+      </c>
+      <c r="N22" s="6">
+        <v>0.12</v>
+      </c>
+      <c r="O22" s="7">
+        <v>0.23</v>
+      </c>
+      <c r="Q22" s="6">
+        <v>7.48</v>
+      </c>
+      <c r="R22" s="6">
+        <v>0.17</v>
+      </c>
+      <c r="S22" s="7">
+        <v>0.34</v>
+      </c>
+      <c r="U22" s="6">
+        <v>5.74</v>
+      </c>
+      <c r="V22" s="6">
+        <v>0.05</v>
+      </c>
+      <c r="W22" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="Y22" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z22" s="6" t="e">
+        <v>7.4224999999999994</v>
+      </c>
+      <c r="Z22" s="6">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA22" s="7" t="e">
+        <v>0.17</v>
+      </c>
+      <c r="AA22" s="7">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>0.33250000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="12"/>
+      <c r="B23" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C23" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" s="1"/>
+      <c r="I23" s="6">
+        <v>8.48</v>
+      </c>
+      <c r="J23" s="6">
+        <v>0.52</v>
+      </c>
+      <c r="K23" s="6">
+        <v>0.99</v>
+      </c>
+      <c r="L23" s="6"/>
+      <c r="M23" s="7">
+        <v>6.67</v>
+      </c>
+      <c r="N23" s="6">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="O23" s="7">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="Q23" s="6">
+        <v>8.3699999999999992</v>
+      </c>
+      <c r="R23" s="6">
+        <v>0.63</v>
+      </c>
+      <c r="S23" s="7">
+        <v>1.17</v>
+      </c>
+      <c r="U23" s="6">
+        <v>5.79</v>
+      </c>
+      <c r="V23" s="6">
+        <v>0.18</v>
+      </c>
+      <c r="W23" s="7">
+        <v>0.36</v>
+      </c>
+      <c r="Y23" s="6">
+        <f t="shared" si="1"/>
+        <v>7.3274999999999997</v>
+      </c>
+      <c r="Z23" s="6">
+        <f t="shared" si="1"/>
+        <v>0.40499999999999997</v>
+      </c>
+      <c r="AA23" s="7">
+        <f t="shared" si="1"/>
+        <v>0.76749999999999996</v>
+      </c>
+      <c r="AB23" s="6"/>
+      <c r="AC23" s="6"/>
+      <c r="AD23" s="6"/>
+      <c r="AE23" s="6"/>
+      <c r="AF23" s="6"/>
+      <c r="AG23" s="6"/>
+      <c r="AH23" s="6"/>
+      <c r="AI23" s="6"/>
+      <c r="AJ23" s="6"/>
+      <c r="AK23" s="6"/>
+      <c r="AL23" s="6"/>
+      <c r="AM23" s="6"/>
+      <c r="AN23" s="6"/>
+      <c r="AO23" s="6"/>
+      <c r="AP23" s="6"/>
+      <c r="AQ23" s="6"/>
+      <c r="AR23" s="6"/>
+    </row>
+    <row r="24" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="12"/>
+      <c r="B24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" s="1"/>
+      <c r="I24" s="6">
+        <v>6.87</v>
+      </c>
+      <c r="J24" s="6">
+        <v>1.07</v>
+      </c>
+      <c r="K24" s="7">
+        <v>1.85</v>
+      </c>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6">
+        <v>2.59</v>
+      </c>
+      <c r="N24" s="6">
+        <v>0.26</v>
+      </c>
+      <c r="O24" s="7">
+        <v>0.47</v>
+      </c>
+      <c r="Q24" s="6">
+        <v>7.99</v>
+      </c>
+      <c r="R24" s="6">
+        <v>1.35</v>
+      </c>
+      <c r="S24" s="7">
+        <v>2.31</v>
+      </c>
+      <c r="U24" s="6">
+        <v>5.46</v>
+      </c>
+      <c r="V24" s="6">
+        <v>0.61</v>
+      </c>
+      <c r="W24" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="Y24" s="6">
+        <f t="shared" si="1"/>
+        <v>5.7275000000000009</v>
+      </c>
+      <c r="Z24" s="6">
+        <f t="shared" si="1"/>
+        <v>0.82250000000000001</v>
+      </c>
+      <c r="AA24" s="7">
+        <f t="shared" si="1"/>
+        <v>1.4325000000000001</v>
+      </c>
+      <c r="AB24" s="6"/>
+      <c r="AC24" s="6"/>
+      <c r="AD24" s="6"/>
+      <c r="AE24" s="6"/>
+      <c r="AF24" s="6"/>
+      <c r="AG24" s="6"/>
+      <c r="AH24" s="6"/>
+      <c r="AI24" s="6"/>
+      <c r="AJ24" s="6"/>
+      <c r="AK24" s="6"/>
+      <c r="AL24" s="6"/>
+      <c r="AM24" s="6"/>
+      <c r="AN24" s="6"/>
+      <c r="AO24" s="6"/>
+      <c r="AP24" s="6"/>
+      <c r="AQ24" s="6"/>
+      <c r="AR24" s="6"/>
+    </row>
+    <row r="25" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" s="1"/>
+      <c r="I25" s="6">
+        <v>8.39</v>
+      </c>
+      <c r="J25" s="6">
+        <v>0.93</v>
+      </c>
+      <c r="K25" s="7">
+        <v>1.68</v>
+      </c>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6">
+        <v>4.24</v>
+      </c>
+      <c r="N25" s="6">
+        <v>0.27</v>
+      </c>
+      <c r="O25" s="7">
+        <v>0.51</v>
+      </c>
+      <c r="Q25" s="6">
+        <v>8.4</v>
+      </c>
+      <c r="R25" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="S25" s="7">
+        <v>1.95</v>
+      </c>
+      <c r="U25" s="6">
+        <v>7.09</v>
+      </c>
+      <c r="V25" s="6">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="W25" s="7">
+        <v>1.05</v>
+      </c>
+      <c r="Y25" s="6">
+        <f t="shared" si="1"/>
+        <v>7.03</v>
+      </c>
+      <c r="Z25" s="6">
+        <f t="shared" si="1"/>
+        <v>0.71750000000000003</v>
+      </c>
+      <c r="AA25" s="7">
+        <f t="shared" si="1"/>
+        <v>1.2974999999999999</v>
+      </c>
+      <c r="AB25" s="6"/>
+      <c r="AC25" s="6"/>
+      <c r="AD25" s="6"/>
+      <c r="AE25" s="6"/>
+      <c r="AF25" s="6"/>
+      <c r="AG25" s="6"/>
+      <c r="AH25" s="6"/>
+      <c r="AI25" s="6"/>
+      <c r="AJ25" s="6"/>
+      <c r="AK25" s="6"/>
+      <c r="AL25" s="6"/>
+      <c r="AM25" s="6"/>
+      <c r="AN25" s="6"/>
+      <c r="AO25" s="6"/>
+      <c r="AP25" s="6"/>
+      <c r="AQ25" s="6"/>
+      <c r="AR25" s="6"/>
+    </row>
     <row r="26" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5647,6 +6313,13 @@
     <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="Y2:AA2"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="M2:O2"/>
+    <mergeCell ref="U2:W2"/>
     <mergeCell ref="AF17:AK17"/>
     <mergeCell ref="AM17:AR17"/>
     <mergeCell ref="I1:K1"/>
@@ -5654,13 +6327,6 @@
     <mergeCell ref="U1:W1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="M1:O1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="Y2:AA2"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="U2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>